<commit_message>
fix: resolve bug in classroom admin page and client
</commit_message>
<xml_diff>
--- a/public/template_file/classroom-template.xlsx
+++ b/public/template_file/classroom-template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zena\Downloads\SMK Web\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\bkt-workspace\SmartKidWeb\smartkids-tvmn\public\template_file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{107904CC-D558-4D5C-90DA-C91EA2A29E6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38ED7463-92E3-4803-B571-DC341DEAE836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7230" yWindow="2895" windowWidth="21195" windowHeight="11295" xr2:uid="{C45C09F7-C0DB-4A67-B73F-5FA2B8001C91}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" xr2:uid="{C45C09F7-C0DB-4A67-B73F-5FA2B8001C91}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,16 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>classname</t>
-  </si>
-  <si>
-    <t>description</t>
-  </si>
-  <si>
-    <t>imageurl</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="6">
   <si>
     <t>Lớp 1</t>
   </si>
@@ -52,6 +43,15 @@
   </si>
   <si>
     <t>https://img.freepik.com/free-vector/girls-boys-students-classroom-with-blackboard_24640-45512.jpg?t=st=1741055695~exp=1741059295~hmac=6870a7403e0beeda151fd8a4df9cedd2fb523f010e95619cb28d8b92fa559155&amp;w=2000</t>
+  </si>
+  <si>
+    <t>Tên lớp học</t>
+  </si>
+  <si>
+    <t>Mô tả</t>
+  </si>
+  <si>
+    <t>Hình ảnh</t>
   </si>
 </sst>
 </file>
@@ -423,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FAE4D71-9076-4F9B-A9AF-BF258ECD770F}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C151"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.42578125" customWidth="1"/>
@@ -433,25 +433,1034 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B15" s="2"/>
+      <c r="C15" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="2"/>
+      <c r="C18" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" t="s">
+        <v>0</v>
+      </c>
+      <c r="B20" s="2"/>
+      <c r="C20" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" t="s">
+        <v>0</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C22" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" t="s">
+        <v>0</v>
+      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" t="s">
+        <v>0</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
+        <v>0</v>
+      </c>
+      <c r="B25" s="2"/>
+      <c r="C25" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" t="s">
+        <v>0</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" t="s">
+        <v>0</v>
+      </c>
+      <c r="B28" s="2"/>
+      <c r="C28" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" t="s">
+        <v>0</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C29" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" t="s">
+        <v>0</v>
+      </c>
+      <c r="B30" s="2"/>
+      <c r="C30" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
+        <v>0</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" t="s">
+        <v>0</v>
+      </c>
+      <c r="B33" s="2"/>
+      <c r="C33" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" t="s">
+        <v>0</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" t="s">
+        <v>0</v>
+      </c>
+      <c r="B35" s="2"/>
+      <c r="C35" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" t="s">
+        <v>0</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
+        <v>0</v>
+      </c>
+      <c r="B38" s="2"/>
+      <c r="C38" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
+        <v>0</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
+        <v>0</v>
+      </c>
+      <c r="B40" s="2"/>
+      <c r="C40" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" t="s">
+        <v>0</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C42" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" t="s">
+        <v>0</v>
+      </c>
+      <c r="B43" s="2"/>
+      <c r="C43" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" t="s">
+        <v>0</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" t="s">
+        <v>0</v>
+      </c>
+      <c r="B45" s="2"/>
+      <c r="C45" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47" t="s">
+        <v>0</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" t="s">
+        <v>0</v>
+      </c>
+      <c r="B48" s="2"/>
+      <c r="C48" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" t="s">
+        <v>0</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C49" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" t="s">
+        <v>0</v>
+      </c>
+      <c r="B50" s="2"/>
+      <c r="C50" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" t="s">
+        <v>0</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C52" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" t="s">
+        <v>0</v>
+      </c>
+      <c r="B53" s="2"/>
+      <c r="C53" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" t="s">
+        <v>0</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" t="s">
+        <v>0</v>
+      </c>
+      <c r="B55" s="2"/>
+      <c r="C55" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" t="s">
+        <v>0</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58" t="s">
+        <v>0</v>
+      </c>
+      <c r="B58" s="2"/>
+      <c r="C58" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" t="s">
+        <v>0</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" t="s">
+        <v>0</v>
+      </c>
+      <c r="B60" s="2"/>
+      <c r="C60" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C62" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B63" s="2"/>
+      <c r="C63" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" t="s">
+        <v>0</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C64" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" t="s">
+        <v>0</v>
+      </c>
+      <c r="B65" s="2"/>
+      <c r="C65" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" t="s">
+        <v>0</v>
+      </c>
+      <c r="B68" s="2"/>
+      <c r="C68" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" t="s">
+        <v>0</v>
+      </c>
+      <c r="B70" s="2"/>
+      <c r="C70" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
+      <c r="A72" t="s">
+        <v>0</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C72" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B73" s="2"/>
+      <c r="C73" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" t="s">
+        <v>0</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C74" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" t="s">
+        <v>0</v>
+      </c>
+      <c r="B75" s="2"/>
+      <c r="C75" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3">
+      <c r="A76" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3">
+      <c r="A77" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B77" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C77" s="1" t="s">
         <v>5</v>
       </c>
+    </row>
+    <row r="78" spans="1:3">
+      <c r="A78" t="s">
+        <v>0</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C78" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3">
+      <c r="A79" t="s">
+        <v>0</v>
+      </c>
+      <c r="B79" s="2"/>
+      <c r="C79" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3">
+      <c r="A80" t="s">
+        <v>0</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C80" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3">
+      <c r="A81" t="s">
+        <v>0</v>
+      </c>
+      <c r="B81" s="2"/>
+      <c r="C81" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3">
+      <c r="A82" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3">
+      <c r="A83" t="s">
+        <v>0</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C83" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3">
+      <c r="A84" t="s">
+        <v>0</v>
+      </c>
+      <c r="B84" s="2"/>
+      <c r="C84" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3">
+      <c r="A85" t="s">
+        <v>0</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C85" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3">
+      <c r="A86" t="s">
+        <v>0</v>
+      </c>
+      <c r="B86" s="2"/>
+      <c r="C86" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3">
+      <c r="A87" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3">
+      <c r="A88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C88" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3">
+      <c r="A89" t="s">
+        <v>0</v>
+      </c>
+      <c r="B89" s="2"/>
+      <c r="C89" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3">
+      <c r="A90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3">
+      <c r="A91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B91" s="2"/>
+      <c r="C91" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3">
+      <c r="A92" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3">
+      <c r="A93" t="s">
+        <v>0</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3">
+      <c r="A94" t="s">
+        <v>0</v>
+      </c>
+      <c r="B94" s="2"/>
+      <c r="C94" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3">
+      <c r="A95" t="s">
+        <v>0</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C95" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3">
+      <c r="A96" t="s">
+        <v>0</v>
+      </c>
+      <c r="B96" s="2"/>
+      <c r="C96" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3">
+      <c r="A97" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3">
+      <c r="A98" t="s">
+        <v>0</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3">
+      <c r="A99" t="s">
+        <v>0</v>
+      </c>
+      <c r="B99" s="2"/>
+      <c r="C99" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3">
+      <c r="A100" t="s">
+        <v>0</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C100" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3">
+      <c r="B101" s="2"/>
+    </row>
+    <row r="103" spans="1:3">
+      <c r="B103" s="2"/>
+    </row>
+    <row r="104" spans="1:3">
+      <c r="B104" s="2"/>
+    </row>
+    <row r="105" spans="1:3">
+      <c r="B105" s="2"/>
+    </row>
+    <row r="106" spans="1:3">
+      <c r="B106" s="2"/>
+    </row>
+    <row r="108" spans="1:3">
+      <c r="B108" s="2"/>
+    </row>
+    <row r="109" spans="1:3">
+      <c r="B109" s="2"/>
+    </row>
+    <row r="110" spans="1:3">
+      <c r="B110" s="2"/>
+    </row>
+    <row r="111" spans="1:3">
+      <c r="B111" s="2"/>
+    </row>
+    <row r="113" spans="2:2">
+      <c r="B113" s="2"/>
+    </row>
+    <row r="114" spans="2:2">
+      <c r="B114" s="2"/>
+    </row>
+    <row r="115" spans="2:2">
+      <c r="B115" s="2"/>
+    </row>
+    <row r="116" spans="2:2">
+      <c r="B116" s="2"/>
+    </row>
+    <row r="118" spans="2:2">
+      <c r="B118" s="2"/>
+    </row>
+    <row r="119" spans="2:2">
+      <c r="B119" s="2"/>
+    </row>
+    <row r="120" spans="2:2">
+      <c r="B120" s="2"/>
+    </row>
+    <row r="121" spans="2:2">
+      <c r="B121" s="2"/>
+    </row>
+    <row r="123" spans="2:2">
+      <c r="B123" s="2"/>
+    </row>
+    <row r="124" spans="2:2">
+      <c r="B124" s="2"/>
+    </row>
+    <row r="125" spans="2:2">
+      <c r="B125" s="2"/>
+    </row>
+    <row r="126" spans="2:2">
+      <c r="B126" s="2"/>
+    </row>
+    <row r="128" spans="2:2">
+      <c r="B128" s="2"/>
+    </row>
+    <row r="129" spans="2:2">
+      <c r="B129" s="2"/>
+    </row>
+    <row r="130" spans="2:2">
+      <c r="B130" s="2"/>
+    </row>
+    <row r="131" spans="2:2">
+      <c r="B131" s="2"/>
+    </row>
+    <row r="133" spans="2:2">
+      <c r="B133" s="2"/>
+    </row>
+    <row r="134" spans="2:2">
+      <c r="B134" s="2"/>
+    </row>
+    <row r="135" spans="2:2">
+      <c r="B135" s="2"/>
+    </row>
+    <row r="136" spans="2:2">
+      <c r="B136" s="2"/>
+    </row>
+    <row r="138" spans="2:2">
+      <c r="B138" s="2"/>
+    </row>
+    <row r="139" spans="2:2">
+      <c r="B139" s="2"/>
+    </row>
+    <row r="140" spans="2:2">
+      <c r="B140" s="2"/>
+    </row>
+    <row r="141" spans="2:2">
+      <c r="B141" s="2"/>
+    </row>
+    <row r="143" spans="2:2">
+      <c r="B143" s="2"/>
+    </row>
+    <row r="144" spans="2:2">
+      <c r="B144" s="2"/>
+    </row>
+    <row r="145" spans="2:2">
+      <c r="B145" s="2"/>
+    </row>
+    <row r="146" spans="2:2">
+      <c r="B146" s="2"/>
+    </row>
+    <row r="148" spans="2:2">
+      <c r="B148" s="2"/>
+    </row>
+    <row r="149" spans="2:2">
+      <c r="B149" s="2"/>
+    </row>
+    <row r="150" spans="2:2">
+      <c r="B150" s="2"/>
+    </row>
+    <row r="151" spans="2:2">
+      <c r="B151" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>